<commit_message>
Group C: C0319 sleeve built from the eight per-size Brennan STEPs (gen_ring CSLEEVE, 9 configurations, closed loop 0 off); decision Q-C-M1 recorded
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BTgFx1CWdETVwpvBapj9nJ
</commit_message>
<xml_diff>
--- a/tools/_out/groupC_20261021/stage/04_DESIGN_TABLES/DesignTable_C0319.xlsx
+++ b/tools/_out/groupC_20261021/stage/04_DESIGN_TABLES/DesignTable_C0319.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:AD11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,117 +430,147 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>H@DRIVE</t>
+          <t>NOSER@DRIVE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COLLARD@DRIVE</t>
+          <t>BORER@DRIVE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>BORE@DRIVE</t>
+          <t>GROOVER@DRIVE</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NOSED@DRIVE</t>
+          <t>COLLARR@DRIVE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>GROOVED@DRIVE</t>
+          <t>SPIGOTR@DRIVE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>REARIR@DRIVE</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>APEXR@DRIVE</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>STEPR@DRIVE</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>TAILR@DRIVE</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>APEXX@DRIVE</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>GROOVEX@DRIVE</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>CHAMX@DRIVE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>COLLARX@DRIVE</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>SPIGOTD@DRIVE</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>TAILD@DRIVE</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>TAILCH@DRIVE</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>INNERD@DRIVE</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L@REF</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>PMIN@REF</t>
-        </is>
-      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>PMAX@REF</t>
+          <t>SPIGOTX@DRIVE</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>TAILX@DRIVE</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>REARIX@DRIVE</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>BOREX@DRIVE</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>STEPX@DRIVE</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>L@DRIVE</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
           <t>$PRP@PartNo</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>$PRP@Threads</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>$PRP@DataStatus</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>$PRP@AxialSource</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>$COMMENT</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>$PRP@ScopeAction</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>$PRP@OMiSKU</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>$PRP@DimSource</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>$PRP@BrennanRecord</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>$PRP@TubeOD</t>
         </is>
       </c>
     </row>
@@ -551,90 +581,110 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1275</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1425</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.1835</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.15486</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.17707</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.15166</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.02068</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.02782</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.05482</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.2045</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.33838</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.22974</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.04716</v>
+      </c>
+      <c r="T3" t="n">
         <v>0.363</v>
       </c>
-      <c r="C3" t="n">
-        <v>0.367</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.255</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.285</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.312</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.303</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.268</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.156</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.161</v>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>C0319-04</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>7/16-20 UNF</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-04 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-04.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:+0.0008 M:-0.0018 C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Brennan record C0319-04: DN=04 OD=0.25000000 A=0.255 C=0.367 H=0.363 A1=0.255 B=0.275 C1=0.367 D=0.312 D1=0.303 E=0.268 G=0.027 H1=0.363 K=0.025 L=0.109 M=0.049 N=0.285 PMIN=0.156 PMAX=0.161</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>C0319-04</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>C0319-04</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>1/4</t>
         </is>
       </c>
     </row>
@@ -645,90 +695,110 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1965</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.21864</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.23957</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.21566</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.02222</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.02778</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.05482</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.2135</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.2395</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.36838</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.24374</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.04716</v>
+      </c>
+      <c r="T4" t="n">
         <v>0.393</v>
       </c>
-      <c r="C4" t="n">
-        <v>0.492</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.418</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.431</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.393</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.151</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.156</v>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>C0319-06</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>9/16-18 UNF</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-06 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-06.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:-0.0012 M:-0.0018 C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Brennan record C0319-06: DN=06 OD=0.37500000 A=0.380 C=0.492 H=0.393 A1=0.380 B=0.400 C1=0.492 D=0.440 D1=0.431 E=0.393 G=0.029 H1=0.393 K=0.025 L=0.125 M=0.049 N=0.418 PMIN=0.151 PMAX=0.156</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>C0319-06</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>C0319-06</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>3/8</t>
         </is>
       </c>
     </row>
@@ -739,90 +809,110 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>0.2675</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.2525</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.2775</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3315</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2935</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2605</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.29578</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.32456</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.28829</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.03371</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.04426</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.07627</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.39946</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.23714</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="T5" t="n">
         <v>0.429</v>
       </c>
-      <c r="C5" t="n">
-        <v>0.663</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.505</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.535</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.555</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.044</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.587</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.577</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.521</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.162</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>C0319-08</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>3/4-16 UNF</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-08 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-08.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:= M:= C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Brennan record C0319-08: DN=08 OD=0.50000000 A=0.505 C=0.663 H=0.429 A1=0.505 B=0.535 C1=0.663 D=0.587 D1=0.577 E=0.521 G=0.044 H1=0.429 K=0.030 L=0.162 M=0.068 N=0.555 PMIN=0.240 PMAX=0.260</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>C0319-08</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>C0319-08</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>1/2</t>
         </is>
       </c>
     </row>
@@ -833,90 +923,110 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>0.3305</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.3155</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.3405</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.3565</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.3235</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.3575</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.38357</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.35129</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.03217</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.04199</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.07091</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.1715</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.41246</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.23114</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.06325</v>
+      </c>
+      <c r="T6" t="n">
         <v>0.442</v>
       </c>
-      <c r="C6" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.631</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.661</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.681</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.713</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.703</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.647</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.227</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.247</v>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>C0319-10</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>7/8-14 UNF</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-10 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-10.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:= M:-0.0008 C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
         <is>
           <t>Brennan record C0319-10: DN=10 OD=0.62500000 A=0.631 C=0.780 H=0.442 A1=0.631 B=0.661 C1=0.780 D=0.713 D1=0.703 E=0.647 G=0.042 H1=0.442 K=0.030 L=0.181 M=0.064 N=0.681 PMIN=0.227 PMAX=0.247</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>C0319-10</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>C0319-10</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>5/8</t>
         </is>
       </c>
     </row>
@@ -927,90 +1037,110 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>0.393</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4035</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.4625</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.42514</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.45607</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.41379</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.0383</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.0508</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.08283</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.1715</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.44546</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.26414</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.07517</v>
+      </c>
+      <c r="T7" t="n">
         <v>0.475</v>
       </c>
-      <c r="C7" t="n">
-        <v>0.925</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.756</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.786</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.8070000000000001</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.838</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.828</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.772</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="P7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>C0319-12</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>1-1/16-12 UN</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-12 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-12.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:+0.0008 M:-0.0008 C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
         <is>
           <t>Brennan record C0319-12: DN=12 OD=0.75000000 A=0.756 C=0.925 H=0.475 A1=0.756 B=0.786 C1=0.925 D=0.838 D1=0.828 E=0.772 G=0.050 H1=0.475 K=0.030 L=0.181 M=0.076 N=0.807 PMIN=0.250 PMAX=0.270</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>C0319-12</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>C0319-12</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>3/4</t>
         </is>
       </c>
     </row>
@@ -1021,90 +1151,110 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5935</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.55271</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.58707</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.53879</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.04137</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.05563</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.08998</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.1715</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.44546</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.25814</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.08232</v>
+      </c>
+      <c r="T8" t="n">
         <v>0.475</v>
       </c>
-      <c r="C8" t="n">
-        <v>1.187</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1.006</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1.036</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.056</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1.088</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1.078</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L8" t="n">
-        <v>1.022</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.244</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.264</v>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>C0319-16</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>1-5/16-12 UN</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-16 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-16.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:+0.0016 M:-0.0007 C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
         <is>
           <t>Brennan record C0319-16: DN=16 OD=1.00000000 A=1.006 C=1.187 H=0.475 A1=1.006 B=1.036 C1=1.187 D=1.088 D1=1.078 E=1.022 G=0.054 H1=0.475 K=0.030 L=0.187 M=0.083 N=1.056 PMIN=0.244 PMAX=0.264</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>C0319-16</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="AB8" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>C0319-16</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1115,90 +1265,110 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>0.6445</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.6545</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.723</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.6705</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.6375</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.68435</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.71415</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.66529</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.04749</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.06473</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.09354999999999999</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.44546</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.26001</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="T9" t="n">
         <v>0.475</v>
       </c>
-      <c r="C9" t="n">
-        <v>1.446</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="E9" t="n">
-        <v>1.289</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1.309</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1.341</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1.331</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L9" t="n">
-        <v>1.275</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.225</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>C0319-20</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>1-5/8-12 UN</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-20 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-20.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:+0.0027 M:= C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
         <is>
           <t>Brennan record C0319-20: DN=20 OD=1.25000000 A=1.260 C=1.446 H=0.475 A1=1.260 B=1.289 C1=1.446 D=1.341 D1=1.331 E=1.275 G=0.062 H1=0.475 K=0.030 L=0.187 M=0.083 N=1.309 PMIN=0.225 PMAX=0.245</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>C0319-20</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="AB9" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>C0319-20</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
         </is>
       </c>
     </row>
@@ -1209,90 +1379,110 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>0.7695</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.7795</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.795</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.80935</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.84057</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.78979</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.04749</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.06473</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.09236</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.44546</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.26188</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.0847</v>
+      </c>
+      <c r="T10" t="n">
         <v>0.475</v>
       </c>
-      <c r="C10" t="n">
-        <v>1.694</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1.539</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1.559</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1.524</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.225</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="P10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>C0319-24</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>1-7/8-12 UN</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-24 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-24.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:+0.0027 M:-0.0013 C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>Brennan record C0319-24: DN=24 OD=1.50000000 A=1.510 C=1.694 H=0.475 A1=1.510 B=1.539 C1=1.694 D=1.590 D1=1.580 E=1.524 G=0.062 H1=0.475 K=0.030 L=0.187 M=0.086 N=1.559 PMIN=0.225 PMAX=0.245</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>C0319-24</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="AB10" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>C0319-24</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>1 1/2</t>
         </is>
       </c>
     </row>
@@ -1303,90 +1493,110 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>1.0195</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.007</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.0475</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.105</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.047</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.013</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.0645</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1.0967</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.04179</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.05362</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.06344</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.10189</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.47946</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0.29961</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="T11" t="n">
         <v>0.509</v>
       </c>
-      <c r="C11" t="n">
-        <v>2.21</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2.014</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2.039</v>
-      </c>
-      <c r="F11" t="n">
-        <v>2.095</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.092</v>
-      </c>
-      <c r="I11" t="n">
-        <v>2.094</v>
-      </c>
-      <c r="J11" t="n">
-        <v>2.084</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L11" t="n">
-        <v>2.026</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.238</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.258</v>
-      </c>
-      <c r="P11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>C0319-32</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>2-1/2-12 UN</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>[BRENNAN-CAD 2026-10-21: every dimension cell] Brennan CAD parameter record C0319-32 (flareless_bite_type_fittings/c0319, PARTcommunity reversemap, exact match) - single source (no Air-Way compression series; OMi file prints threads only)</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>[BRENNAN-STEP 2026-10-21: every DRIVE cell measured on BRENNAN_C0319-32.stp] Brennan 3D model of the part (user upload 2026-10-21, PARTcommunity) - single source (no Air-Way compression series; OMi file prints threads only); the 14-line half-section read by groupC scripts/measure_c0319.py; Brennan record letters vs the STEP: A:= B:= N:= G:-0.0066 M:= C:= D:= D1:= E:= H:= K:= (G / M are not exactly the groove start / end on the STEP - the STEP is used)</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Brennan record C0319-32: DN=32 OD=2.00000000 A=2.014 C=2.210 H=0.509 A1=2.014 B=2.039 C1=2.210 D=2.094 D1=2.084 E=2.026 G=0.070 H1=0.509 K=0.030 L=0.187 M=0.092 N=2.095 PMIN=0.238 PMAX=0.258</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>C0319-32</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="AB11" t="inlineStr">
         <is>
           <t>BRENNAN</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>C0319-32</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>